<commit_message>
Updated excel import service with better validations
</commit_message>
<xml_diff>
--- a/ApplicationRecords_Import_Template.xlsx
+++ b/ApplicationRecords_Import_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\FullStackProject\ApplicationTracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4757DF04-0071-4484-BCFF-F44E88A8D0F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{456525B2-A7DF-4F36-B214-97DF6716D93B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3690" yWindow="5085" windowWidth="28800" windowHeight="15435" xr2:uid="{0DC61EF3-0AB4-4D72-BBD1-F2775F03C231}"/>
+    <workbookView xWindow="-38520" yWindow="-60" windowWidth="38640" windowHeight="21240" xr2:uid="{0DC61EF3-0AB4-4D72-BBD1-F2775F03C231}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -421,7 +421,7 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D1" t="s">

</xml_diff>

<commit_message>
Updated import file template
</commit_message>
<xml_diff>
--- a/ApplicationRecords_Import_Template.xlsx
+++ b/ApplicationRecords_Import_Template.xlsx
@@ -676,7 +676,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1">
+    <row r="8" ht="60" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>AppliedDate (C)</t>
@@ -689,17 +689,20 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>YYYY-MM-DD  (e.g. 2026-06-17)</t>
+          <t>YYYY-MM-DD (recommended)
+MM/DD/YYYY
+YYYY/MM/DD
+MMM D, YYYY (e.g. Jun 18, 2026)</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Future dates are rejected. Leave no time component.</t>
+          <t>Multiple formats accepted; YYYY-MM-DD is least ambiguous. Future dates are rejected.</t>
         </is>
       </c>
     </row>

</xml_diff>